<commit_message>
Updating and Deleting an Excel file
</commit_message>
<xml_diff>
--- a/DDT_JAVA/TestData.xlsx
+++ b/DDT_JAVA/TestData.xlsx
@@ -5,14 +5,12 @@
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
-  <sheets>
-    <sheet name="TestDataSheet" r:id="rId3" sheetId="1"/>
-  </sheets>
+  <sheets/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Name</t>
   </si>
@@ -27,6 +25,33 @@
   </si>
   <si>
     <t>New York</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Maria Rossi</t>
+  </si>
+  <si>
+    <t>Frankfurt</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Alice Smith</t>
+  </si>
+  <si>
+    <t>Los Angeles</t>
+  </si>
+  <si>
+    <t>Canada</t>
   </si>
 </sst>
 </file>
@@ -67,47 +92,4 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
 </styleSheet>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B2" t="n" s="0">
-        <v>30.0</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B3" t="n" s="0">
-        <v>30.0</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
 </file>
</xml_diff>